<commit_message>
Atualizando pós-jogo do Brasil
</commit_message>
<xml_diff>
--- a/planilhas_competidores/Bruno_previsoes.xlsx
+++ b/planilhas_competidores/Bruno_previsoes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BIEL\bolao-copa-2026\planilhas_competidores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6605188-3911-4960-BF53-A977CCC40A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35EDBEDC-C4C9-4355-B0E3-C04A09E902DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10140" yWindow="0" windowWidth="10455" windowHeight="11625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10035" yWindow="0" windowWidth="10455" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -855,7 +855,7 @@
         <v>2</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -1026,10 +1026,10 @@
         <v>34</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I10">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -1055,7 +1055,7 @@
         <v>36</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I11">
         <v>1</v>
@@ -1200,7 +1200,7 @@
         <v>44</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I16">
         <v>2</v>
@@ -1229,7 +1229,7 @@
         <v>46</v>
       </c>
       <c r="H17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I17">
         <v>0</v>
@@ -1374,10 +1374,10 @@
         <v>37</v>
       </c>
       <c r="H22">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I22">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -1403,10 +1403,10 @@
         <v>56</v>
       </c>
       <c r="H23">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I23">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -2170,7 +2170,7 @@
         <v>1</v>
       </c>
       <c r="I51">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -2315,7 +2315,7 @@
         <v>4</v>
       </c>
       <c r="I56">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -2344,7 +2344,7 @@
         <v>1</v>
       </c>
       <c r="I57">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -2486,10 +2486,10 @@
         <v>62</v>
       </c>
       <c r="H62">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I62">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -2515,10 +2515,10 @@
         <v>14</v>
       </c>
       <c r="H63">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I63">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -2663,7 +2663,7 @@
         <v>2</v>
       </c>
       <c r="I68">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -2689,7 +2689,7 @@
         <v>29</v>
       </c>
       <c r="H69">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I69">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização com resultados de 22/06/26
</commit_message>
<xml_diff>
--- a/planilhas_competidores/Bruno_previsoes.xlsx
+++ b/planilhas_competidores/Bruno_previsoes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BIEL\bolao-copa-2026\planilhas_competidores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5C9CBBE-58C3-4DFC-B416-85526375C05E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF32DFB-DC08-4A22-B1C2-6A47AFA81992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10035" yWindow="0" windowWidth="10455" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2220,7 +2220,7 @@
         <v>46</v>
       </c>
       <c r="H52">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I52">
         <v>0</v>
@@ -2249,7 +2249,7 @@
         <v>41</v>
       </c>
       <c r="H53">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I53">
         <v>1</v>

</xml_diff>